<commit_message>
camioneros: escala de septiembre 2026 a febrero 2027 desde las planillas firmadas de FADEEAC
Acuerdo del 18/9/2026 (Disp. DNRyRT 1277/2026): seis meses nuevos con las 9 categorías,
cruzadas contra la columna por día y con salto uniforme entre categorías. Octubre se deriva
como septiembre x 1,017 + $12.252,86 incorporados (cláusula PRIMERA) y el check lo exige.
Homologación por mes en /convenios/camioneros/[mes], viáticos de octubre en la planilla paga,
asignación extraordinaria de enero-abril 2027 en fuentes y FAQ.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/private/planilla-camioneros-2026.xlsx
+++ b/private/planilla-camioneros-2026.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="211" uniqueCount="188">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="242" uniqueCount="214">
   <si>
     <t>Planilla de sueldos Camioneros 2026 — cómo usarla</t>
   </si>
@@ -64,7 +64,7 @@
     <t>LO QUE TENÉS QUE SABER DEL CCT 40/89</t>
   </si>
   <si>
-    <t>•  Escala nacional única: el básico es el mismo en todo el país. Los básicos de esta planilla son los de las planillas firmadas que publica FADEEAC, de marzo 2026 a agosto 2026 (Disposición DNRyRT 455/2026 y revisión de julio).</t>
+    <t>•  Escala nacional única: el básico es el mismo en todo el país. Los básicos de esta planilla son los de las planillas firmadas que publica FADEEAC, de marzo 2026 a febrero 2027 (Disposiciones DNRyRT 455/2026 y 1277/2026, y revisión de julio).</t>
   </si>
   <si>
     <t>•  Antigüedad (ítem 6.1.5): 1% por año sobre los conceptos remunerativos. Sin kilómetros ni adicionales, es el 1% del básico por año.</t>
@@ -79,13 +79,13 @@
     <t>•  Zona: quien reside al sur del Río Colorado cobra los viáticos y el 4.2.3 con coeficiente 1,2, y al sur del Río Santa Cruz con 1,4. El básico no cambia.</t>
   </si>
   <si>
-    <t>•  Los valores de viáticos son los de la planilla de agosto 2026. Si liquidás otro mes, reemplazalos en el Liquidador por los de esa planilla (son celdas amarillas).</t>
+    <t>•  Los valores de viáticos son los de la planilla de octubre 2026. Si liquidás otro mes, reemplazalos en el Liquidador por los de esa planilla (son celdas amarillas).</t>
   </si>
   <si>
     <t>•  Aportes del trabajador: 11% jubilación, 3% PAMI (Ley 19.032) y 3% obra social, sobre lo remunerativo.</t>
   </si>
   <si>
-    <t>•  La escala de septiembre de 2026 a febrero de 2027 ya está acordada (FADEEAC publicó la homologación, Disposición 1277/26), pero las planillas firmadas de cada mes todavía no salieron. Apenas FADEEAC las publique, las cargamos y la versión nueva te llega al mismo enlace de descarga: no vence.</t>
+    <t>•  La escala llega hasta febrero 2027, la última planilla firmada publicada por FADEEAC. Cuando salga la siguiente, la cargamos y la versión nueva te llega al mismo enlace de descarga: no vence.</t>
   </si>
   <si>
     <t>Es una referencia de cálculo con las fuentes a la vista, no un recibo oficial. No incluye contribuciones patronales, ART, cuota sindical ni aportes solidarios del convenio, Ganancias ni embargos. Los adicionales por rama (combustibles, sustancias peligrosas, larga distancia y otros) se cargan en «Otros adicionales».</t>
@@ -97,7 +97,7 @@
     <t>Liquidación de sueldo — Camioneros (CCT 40/89)</t>
   </si>
   <si>
-    <t>Básicos de las planillas firmadas FADEEAC · verificados el 20/09/2026 · calcular.ar</t>
+    <t>Básicos de las planillas firmadas FADEEAC · verificados el 10/10/2026 · calcular.ar</t>
   </si>
   <si>
     <t>DATOS DEL TRABAJADOR</t>
@@ -112,340 +112,358 @@
     <t>Mes a liquidar</t>
   </si>
   <si>
+    <t>Febrero 2027</t>
+  </si>
+  <si>
+    <t>Años de antigüedad</t>
+  </si>
+  <si>
+    <t>Ítem 6.1.5: 1% por año sobre lo remunerativo</t>
+  </si>
+  <si>
+    <t>Zona de residencia</t>
+  </si>
+  <si>
+    <t>General</t>
+  </si>
+  <si>
+    <t>Coeficiente 1,20 / 1,40 sobre viáticos y 4.2.3</t>
+  </si>
+  <si>
+    <t>VIAJES Y ADICIONALES DEL MES (en cero si no viajó)</t>
+  </si>
+  <si>
+    <t>Km recorridos — horas extra por km</t>
+  </si>
+  <si>
+    <t>Ítem 4.2.3 · remunerativo</t>
+  </si>
+  <si>
+    <t>Km recorridos — viático por km</t>
+  </si>
+  <si>
+    <t>Ítem 4.2.4 · no remunerativo · mínimo 350 km por día de viaje</t>
+  </si>
+  <si>
+    <t>Comidas</t>
+  </si>
+  <si>
+    <t>Ítem 4.1.12 · no remunerativo</t>
+  </si>
+  <si>
+    <t>Viáticos especiales</t>
+  </si>
+  <si>
+    <t>Ítem 4.1.13 · no remunerativo</t>
+  </si>
+  <si>
+    <t>Pernoctadas</t>
+  </si>
+  <si>
+    <t>Ítem 4.1.14 · no remunerativo</t>
+  </si>
+  <si>
+    <t>Otros adicionales remunerativos ($)</t>
+  </si>
+  <si>
+    <t>Adicionales por rama, horas extra, etc.</t>
+  </si>
+  <si>
+    <t>Otros no remunerativos ($)</t>
+  </si>
+  <si>
+    <t>Permanencia (4.2.5), cruce de frontera (4.2.17), etc.</t>
+  </si>
+  <si>
+    <t>LIQUIDACIÓN DEL MES</t>
+  </si>
+  <si>
+    <t>Sueldo básico</t>
+  </si>
+  <si>
+    <t>Horas extra por km (4.2.3)</t>
+  </si>
+  <si>
+    <t>Otros adicionales remunerativos</t>
+  </si>
+  <si>
+    <t>Antigüedad</t>
+  </si>
+  <si>
+    <t>TOTAL REMUNERATIVO (bruto)</t>
+  </si>
+  <si>
+    <t>Base de aportes y del aguinaldo</t>
+  </si>
+  <si>
+    <t>Jubilación (11%)</t>
+  </si>
+  <si>
+    <t>PAMI — Ley 19.032 (3%)</t>
+  </si>
+  <si>
+    <t>Obra social (3%)</t>
+  </si>
+  <si>
+    <t>NETO DE HABERES</t>
+  </si>
+  <si>
+    <t>Viáticos no remunerativos</t>
+  </si>
+  <si>
+    <t>No llevan aportes (ítem 4.2.11 y art. 106 LCT)</t>
+  </si>
+  <si>
+    <t>TOTAL A COBRAR</t>
+  </si>
+  <si>
+    <t>VALORES DE VIÁTICOS (planilla octubre 2026)</t>
+  </si>
+  <si>
+    <t>Valor por km (4.2.3 y 4.2.4)</t>
+  </si>
+  <si>
+    <t>Comida (4.1.12)</t>
+  </si>
+  <si>
+    <t>Viático especial (4.1.13)</t>
+  </si>
+  <si>
+    <t>Pernoctada (4.1.14)</t>
+  </si>
+  <si>
+    <t>* El sueldo del convenio es un piso: si pagan más, cargá la diferencia en «Otros adicionales remunerativos».</t>
+  </si>
+  <si>
+    <t>* El neto no descuenta cuota sindical, aportes solidarios, Ganancias ni embargos. No incluye contribuciones patronales ni ART.</t>
+  </si>
+  <si>
+    <t>* Las celdas amarillas se completan; las verdes las calcula la planilla. La columna D está oculta a propósito: no la borres.</t>
+  </si>
+  <si>
+    <t>Nómina del mes — toda la flota en una hoja</t>
+  </si>
+  <si>
+    <t>Mes liquidado</t>
+  </si>
+  <si>
+    <t>El mes y los valores de viáticos salen del Liquidador. Un trabajador por fila; las filas sin categoría no suman.</t>
+  </si>
+  <si>
+    <t>Amarillo: lo cargás vos. Verde: lo calcula la planilla. Con km y viáticos en cero, cada fila da lo mismo que la calculadora gratis.</t>
+  </si>
+  <si>
+    <t>Trabajador</t>
+  </si>
+  <si>
+    <t>Años</t>
+  </si>
+  <si>
+    <t>Zona</t>
+  </si>
+  <si>
+    <t>Km 4.2.3</t>
+  </si>
+  <si>
+    <t>Km 4.2.4</t>
+  </si>
+  <si>
+    <t>Viát. esp.</t>
+  </si>
+  <si>
+    <t>Pernoct.</t>
+  </si>
+  <si>
+    <t>Otros rem. $</t>
+  </si>
+  <si>
+    <t>Otros no rem. $</t>
+  </si>
+  <si>
+    <t>Básico</t>
+  </si>
+  <si>
+    <t>Horas extra km</t>
+  </si>
+  <si>
+    <t>Total remunerativo</t>
+  </si>
+  <si>
+    <t>Aportes 17%</t>
+  </si>
+  <si>
+    <t>Neto de haberes</t>
+  </si>
+  <si>
+    <t>No remunerativo</t>
+  </si>
+  <si>
+    <t>A cobrar</t>
+  </si>
+  <si>
+    <t>coef</t>
+  </si>
+  <si>
+    <t>Trabajador 1</t>
+  </si>
+  <si>
+    <t>TOTALES DEL MES</t>
+  </si>
+  <si>
+    <t>Recibo de haberes — CCT 40/89 Camioneros</t>
+  </si>
+  <si>
+    <t>Se completa solo con el Liquidador. Los datos de la empresa y del trabajador se escriben una vez acá: no salen de tu computadora.</t>
+  </si>
+  <si>
+    <t>Empleador (razón social)</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>CUIT del empleador</t>
+  </si>
+  <si>
+    <t>Trabajador (apellido y nombre)</t>
+  </si>
+  <si>
+    <t>CUIL del trabajador</t>
+  </si>
+  <si>
+    <t>Fecha de ingreso</t>
+  </si>
+  <si>
+    <t>Período</t>
+  </si>
+  <si>
+    <t>Concepto</t>
+  </si>
+  <si>
+    <t>Cantidad</t>
+  </si>
+  <si>
+    <t>Haberes rem.</t>
+  </si>
+  <si>
+    <t>Descuentos</t>
+  </si>
+  <si>
+    <t>Antigüedad (6.1.5)</t>
+  </si>
+  <si>
+    <t>Viáticos, comidas y pernoctadas (no rem.)</t>
+  </si>
+  <si>
+    <t>Jubilación 11%</t>
+  </si>
+  <si>
+    <t>PAMI Ley 19.032 3%</t>
+  </si>
+  <si>
+    <t>Obra social 3%</t>
+  </si>
+  <si>
+    <t>Totales</t>
+  </si>
+  <si>
+    <t>NETO A COBRAR</t>
+  </si>
+  <si>
+    <t>Lugar y fecha de pago</t>
+  </si>
+  <si>
+    <t>Los aportes del trabajador se depositaron en el período anterior. Recibí el importe neto de este recibo y un duplicado firmado.</t>
+  </si>
+  <si>
+    <t>Firma del trabajador</t>
+  </si>
+  <si>
+    <t>Firma y sello del empleador</t>
+  </si>
+  <si>
+    <t>Aguinaldo (SAC) — Ley 23.041 y arts. 121 a 123 LCT</t>
+  </si>
+  <si>
+    <t>DATOS DEL SEMESTRE</t>
+  </si>
+  <si>
+    <t>Semestre</t>
+  </si>
+  <si>
+    <t>2do semestre 2026</t>
+  </si>
+  <si>
+    <t>Vienen con el bruto del Liquidador: escribí encima lo que pagaste cada mes</t>
+  </si>
+  <si>
+    <t>Días trabajados en el semestre</t>
+  </si>
+  <si>
+    <t>Dejala vacía si trabajó el semestre completo</t>
+  </si>
+  <si>
+    <t>AGUINALDO</t>
+  </si>
+  <si>
+    <t>Mejor remuneración del semestre</t>
+  </si>
+  <si>
+    <t>Días del semestre</t>
+  </si>
+  <si>
+    <t>Días computados</t>
+  </si>
+  <si>
+    <t>SAC bruto</t>
+  </si>
+  <si>
+    <t>PAMI (3%)</t>
+  </si>
+  <si>
+    <t>SAC NETO ESTIMADO</t>
+  </si>
+  <si>
+    <t>* El aguinaldo es el 50% de la MEJOR remuneración mensual del semestre, no el promedio. Si trabajó una parte, es proporcional a los días.</t>
+  </si>
+  <si>
+    <t>* Vencimientos: 30 de junio de 2026 y 18 de diciembre de 2026 (art. 122 LCT). Los viáticos no remunerativos (4.1.12, 4.1.13, 4.1.14, 4.2.4) no entran en la base.</t>
+  </si>
+  <si>
+    <t>Básicos mensuales oficiales — CCT 40/89 (planillas firmadas FADEEAC)</t>
+  </si>
+  <si>
+    <t>Marzo 2026</t>
+  </si>
+  <si>
+    <t>Abril 2026</t>
+  </si>
+  <si>
+    <t>Mayo 2026</t>
+  </si>
+  <si>
+    <t>Junio 2026</t>
+  </si>
+  <si>
+    <t>Julio 2026</t>
+  </si>
+  <si>
     <t>Agosto 2026</t>
   </si>
   <si>
-    <t>Años de antigüedad</t>
-  </si>
-  <si>
-    <t>Ítem 6.1.5: 1% por año sobre lo remunerativo</t>
-  </si>
-  <si>
-    <t>Zona de residencia</t>
-  </si>
-  <si>
-    <t>General</t>
-  </si>
-  <si>
-    <t>Coeficiente 1,20 / 1,40 sobre viáticos y 4.2.3</t>
-  </si>
-  <si>
-    <t>VIAJES Y ADICIONALES DEL MES (en cero si no viajó)</t>
-  </si>
-  <si>
-    <t>Km recorridos — horas extra por km</t>
-  </si>
-  <si>
-    <t>Ítem 4.2.3 · remunerativo</t>
-  </si>
-  <si>
-    <t>Km recorridos — viático por km</t>
-  </si>
-  <si>
-    <t>Ítem 4.2.4 · no remunerativo · mínimo 350 km por día de viaje</t>
-  </si>
-  <si>
-    <t>Comidas</t>
-  </si>
-  <si>
-    <t>Ítem 4.1.12 · no remunerativo</t>
-  </si>
-  <si>
-    <t>Viáticos especiales</t>
-  </si>
-  <si>
-    <t>Ítem 4.1.13 · no remunerativo</t>
-  </si>
-  <si>
-    <t>Pernoctadas</t>
-  </si>
-  <si>
-    <t>Ítem 4.1.14 · no remunerativo</t>
-  </si>
-  <si>
-    <t>Otros adicionales remunerativos ($)</t>
-  </si>
-  <si>
-    <t>Adicionales por rama, horas extra, etc.</t>
-  </si>
-  <si>
-    <t>Otros no remunerativos ($)</t>
-  </si>
-  <si>
-    <t>Permanencia (4.2.5), cruce de frontera (4.2.17), etc.</t>
-  </si>
-  <si>
-    <t>LIQUIDACIÓN DEL MES</t>
-  </si>
-  <si>
-    <t>Sueldo básico</t>
-  </si>
-  <si>
-    <t>Horas extra por km (4.2.3)</t>
-  </si>
-  <si>
-    <t>Otros adicionales remunerativos</t>
-  </si>
-  <si>
-    <t>Antigüedad</t>
-  </si>
-  <si>
-    <t>TOTAL REMUNERATIVO (bruto)</t>
-  </si>
-  <si>
-    <t>Base de aportes y del aguinaldo</t>
-  </si>
-  <si>
-    <t>Jubilación (11%)</t>
-  </si>
-  <si>
-    <t>PAMI — Ley 19.032 (3%)</t>
-  </si>
-  <si>
-    <t>Obra social (3%)</t>
-  </si>
-  <si>
-    <t>NETO DE HABERES</t>
-  </si>
-  <si>
-    <t>Viáticos no remunerativos</t>
-  </si>
-  <si>
-    <t>No llevan aportes (ítem 4.2.11 y art. 106 LCT)</t>
-  </si>
-  <si>
-    <t>TOTAL A COBRAR</t>
-  </si>
-  <si>
-    <t>VALORES DE VIÁTICOS (planilla agosto 2026)</t>
-  </si>
-  <si>
-    <t>Valor por km (4.2.3 y 4.2.4)</t>
-  </si>
-  <si>
-    <t>Comida (4.1.12)</t>
-  </si>
-  <si>
-    <t>Viático especial (4.1.13)</t>
-  </si>
-  <si>
-    <t>Pernoctada (4.1.14)</t>
-  </si>
-  <si>
-    <t>* El sueldo del convenio es un piso: si pagan más, cargá la diferencia en «Otros adicionales remunerativos».</t>
-  </si>
-  <si>
-    <t>* El neto no descuenta cuota sindical, aportes solidarios, Ganancias ni embargos. No incluye contribuciones patronales ni ART.</t>
-  </si>
-  <si>
-    <t>* Las celdas amarillas se completan; las verdes las calcula la planilla. La columna D está oculta a propósito: no la borres.</t>
-  </si>
-  <si>
-    <t>Nómina del mes — toda la flota en una hoja</t>
-  </si>
-  <si>
-    <t>Mes liquidado</t>
-  </si>
-  <si>
-    <t>El mes y los valores de viáticos salen del Liquidador. Un trabajador por fila; las filas sin categoría no suman.</t>
-  </si>
-  <si>
-    <t>Amarillo: lo cargás vos. Verde: lo calcula la planilla. Con km y viáticos en cero, cada fila da lo mismo que la calculadora gratis.</t>
-  </si>
-  <si>
-    <t>Trabajador</t>
-  </si>
-  <si>
-    <t>Años</t>
-  </si>
-  <si>
-    <t>Zona</t>
-  </si>
-  <si>
-    <t>Km 4.2.3</t>
-  </si>
-  <si>
-    <t>Km 4.2.4</t>
-  </si>
-  <si>
-    <t>Viát. esp.</t>
-  </si>
-  <si>
-    <t>Pernoct.</t>
-  </si>
-  <si>
-    <t>Otros rem. $</t>
-  </si>
-  <si>
-    <t>Otros no rem. $</t>
-  </si>
-  <si>
-    <t>Básico</t>
-  </si>
-  <si>
-    <t>Horas extra km</t>
-  </si>
-  <si>
-    <t>Total remunerativo</t>
-  </si>
-  <si>
-    <t>Aportes 17%</t>
-  </si>
-  <si>
-    <t>Neto de haberes</t>
-  </si>
-  <si>
-    <t>No remunerativo</t>
-  </si>
-  <si>
-    <t>A cobrar</t>
-  </si>
-  <si>
-    <t>coef</t>
-  </si>
-  <si>
-    <t>Trabajador 1</t>
-  </si>
-  <si>
-    <t>TOTALES DEL MES</t>
-  </si>
-  <si>
-    <t>Recibo de haberes — CCT 40/89 Camioneros</t>
-  </si>
-  <si>
-    <t>Se completa solo con el Liquidador. Los datos de la empresa y del trabajador se escriben una vez acá: no salen de tu computadora.</t>
-  </si>
-  <si>
-    <t>Empleador (razón social)</t>
-  </si>
-  <si>
-    <t/>
-  </si>
-  <si>
-    <t>CUIT del empleador</t>
-  </si>
-  <si>
-    <t>Trabajador (apellido y nombre)</t>
-  </si>
-  <si>
-    <t>CUIL del trabajador</t>
-  </si>
-  <si>
-    <t>Fecha de ingreso</t>
-  </si>
-  <si>
-    <t>Período</t>
-  </si>
-  <si>
-    <t>Concepto</t>
-  </si>
-  <si>
-    <t>Cantidad</t>
-  </si>
-  <si>
-    <t>Haberes rem.</t>
-  </si>
-  <si>
-    <t>Descuentos</t>
-  </si>
-  <si>
-    <t>Antigüedad (6.1.5)</t>
-  </si>
-  <si>
-    <t>Viáticos, comidas y pernoctadas (no rem.)</t>
-  </si>
-  <si>
-    <t>Jubilación 11%</t>
-  </si>
-  <si>
-    <t>PAMI Ley 19.032 3%</t>
-  </si>
-  <si>
-    <t>Obra social 3%</t>
-  </si>
-  <si>
-    <t>Totales</t>
-  </si>
-  <si>
-    <t>NETO A COBRAR</t>
-  </si>
-  <si>
-    <t>Lugar y fecha de pago</t>
-  </si>
-  <si>
-    <t>Los aportes del trabajador se depositaron en el período anterior. Recibí el importe neto de este recibo y un duplicado firmado.</t>
-  </si>
-  <si>
-    <t>Firma del trabajador</t>
-  </si>
-  <si>
-    <t>Firma y sello del empleador</t>
-  </si>
-  <si>
-    <t>Aguinaldo (SAC) — Ley 23.041 y arts. 121 a 123 LCT</t>
-  </si>
-  <si>
-    <t>DATOS DEL SEMESTRE</t>
-  </si>
-  <si>
-    <t>Semestre</t>
-  </si>
-  <si>
-    <t>2do semestre 2026</t>
-  </si>
-  <si>
-    <t>Vienen con el bruto del Liquidador: escribí encima lo que pagaste cada mes</t>
-  </si>
-  <si>
-    <t>Días trabajados en el semestre</t>
-  </si>
-  <si>
-    <t>Dejala vacía si trabajó el semestre completo</t>
-  </si>
-  <si>
-    <t>AGUINALDO</t>
-  </si>
-  <si>
-    <t>Mejor remuneración del semestre</t>
-  </si>
-  <si>
-    <t>Días del semestre</t>
-  </si>
-  <si>
-    <t>Días computados</t>
-  </si>
-  <si>
-    <t>SAC bruto</t>
-  </si>
-  <si>
-    <t>PAMI (3%)</t>
-  </si>
-  <si>
-    <t>SAC NETO ESTIMADO</t>
-  </si>
-  <si>
-    <t>* El aguinaldo es el 50% de la MEJOR remuneración mensual del semestre, no el promedio. Si trabajó una parte, es proporcional a los días.</t>
-  </si>
-  <si>
-    <t>* Vencimientos: 30 de junio de 2026 y 18 de diciembre de 2026 (art. 122 LCT). Los viáticos no remunerativos (4.1.12, 4.1.13, 4.1.14, 4.2.4) no entran en la base.</t>
-  </si>
-  <si>
-    <t>Básicos mensuales oficiales — CCT 40/89 (planillas firmadas FADEEAC)</t>
-  </si>
-  <si>
-    <t>Marzo 2026</t>
-  </si>
-  <si>
-    <t>Abril 2026</t>
-  </si>
-  <si>
-    <t>Mayo 2026</t>
-  </si>
-  <si>
-    <t>Junio 2026</t>
-  </si>
-  <si>
-    <t>Julio 2026</t>
+    <t>Septiembre 2026</t>
+  </si>
+  <si>
+    <t>Octubre 2026</t>
+  </si>
+  <si>
+    <t>Noviembre 2026</t>
+  </si>
+  <si>
+    <t>Diciembre 2026</t>
+  </si>
+  <si>
+    <t>Enero 2027</t>
   </si>
   <si>
     <t>Chofer de Segunda</t>
@@ -487,10 +505,28 @@
     <t>Julio 2026: +4,22% sobre junio: acá entra la REVISIÓN de la cláusula TERCERA (no es el +1,5% del tramo original). La escala de julio se republicó firmada en agosto.</t>
   </si>
   <si>
-    <t>Agosto 2026: Último tramo del acuerdo: +1,5% sobre el básico de julio (ya revisado). La próxima ronda de negociación está pactada para septiembre de 2026.</t>
-  </si>
-  <si>
-    <t>La escala de septiembre de 2026 a febrero de 2027 ya está acordada (FADEEAC publicó la homologación, Disposición 1277/26), pero las planillas firmadas de cada mes todavía no salieron. Apenas FADEEAC las publique, las cargamos y la versión nueva te llega al mismo enlace de descarga: no vence.</t>
+    <t>Agosto 2026: Último tramo del acuerdo: +1,5% sobre el básico de julio (ya revisado). Desde septiembre rige el acuerdo del 18/9/2026.</t>
+  </si>
+  <si>
+    <t>Septiembre 2026: Primer tramo del acuerdo del 18/9/2026: +1,8% sobre el básico de agosto. Además, suma no remunerativa de $18.000 por única vez con los haberes de septiembre (cláusula PRIMERA).</t>
+  </si>
+  <si>
+    <t>Octubre 2026: Tramo de octubre: +1,7% sobre septiembre, y se incorporan al básico $12.252,86 de la suma no remunerativa de septiembre (al Chofer de Primera, y en proporción al resto). En total, +2,82%.</t>
+  </si>
+  <si>
+    <t>Noviembre 2026: Tramo de noviembre: +1,7% sobre el básico de octubre.</t>
+  </si>
+  <si>
+    <t>Diciembre 2026: Tramo de diciembre: +1,6% sobre el básico de noviembre. El acuerdo prevé una revisión en la primera quincena de diciembre contra la inflación de septiembre a noviembre.</t>
+  </si>
+  <si>
+    <t>Enero 2027: Tramo de enero: +1,6% sobre el básico de diciembre. Además, empieza la asignación extraordinaria no remunerativa: 4 cuotas de $300.000 (enero a abril de 2027).</t>
+  </si>
+  <si>
+    <t>Febrero 2027: Último tramo del acuerdo del 18/9/2026: +1,5% sobre el básico de enero. Hay una revisión pactada para la primera quincena de marzo de 2027.</t>
+  </si>
+  <si>
+    <t>La escala llega hasta febrero 2027, la última planilla firmada publicada por FADEEAC. Cuando salga la siguiente, la cargamos y la versión nueva te llega al mismo enlace de descarga: no vence.</t>
   </si>
   <si>
     <t>El Liquidador y la Nómina buscan el básico por el nombre de la categoría y del mes: no los edites.</t>
@@ -499,7 +535,7 @@
     <t>Fuentes oficiales</t>
   </si>
   <si>
-    <t>Todos los datos de esta planilla se verificaron el 20/09/2026 contra los documentos oficiales de abajo. Ningún blog, ningún resumen de terceros.</t>
+    <t>Todos los datos de esta planilla se verificaron el 10/10/2026 contra los documentos oficiales de abajo. Ningún blog, ningún resumen de terceros.</t>
   </si>
   <si>
     <t>Documento</t>
@@ -544,7 +580,28 @@
     <t>https://www.fadeeac.org.ar/wp-content/uploads/2026/08/Planillas-de-escalas-salariales-agosto-2026-OK.pdf</t>
   </si>
   <si>
-    <t>Viáticos y adicionales (hoja 2 de la planilla de agosto 2026) — verificado el 06/10/2026</t>
+    <t>FADEEAC — planilla salarial firmada de septiembre 2026 (CCT 40/89)</t>
+  </si>
+  <si>
+    <t>https://www.fadeeac.org.ar/wp-content/uploads/2026/10/3-Planillas-salariales-acuerdo-SEPT-2026-a-FEB-2027.pdf</t>
+  </si>
+  <si>
+    <t>FADEEAC — planilla salarial firmada de octubre 2026 (CCT 40/89)</t>
+  </si>
+  <si>
+    <t>FADEEAC — planilla salarial firmada de noviembre 2026 (CCT 40/89)</t>
+  </si>
+  <si>
+    <t>FADEEAC — planilla salarial firmada de diciembre 2026 (CCT 40/89)</t>
+  </si>
+  <si>
+    <t>FADEEAC — planilla salarial firmada de enero 2027 (CCT 40/89)</t>
+  </si>
+  <si>
+    <t>FADEEAC — planilla salarial firmada de febrero 2027 (CCT 40/89)</t>
+  </si>
+  <si>
+    <t>Viáticos y adicionales (hoja 2 de la planilla de octubre 2026) — verificado el 10/10/2026</t>
   </si>
   <si>
     <t>Acuerdo paritario del 13/3/2026: CCT 40/89 (marzo a agosto 2026), PDF firmado</t>
@@ -565,6 +622,24 @@
     <t>https://www.fadeeac.org.ar/wp-content/uploads/2026/08/REVISION-Acuerdo-Julio-Agosto-2026.pdf</t>
   </si>
   <si>
+    <t>Acuerdo paritario del 18/9/2026: CCT 40/89 (septiembre 2026 a febrero 2027), PDF firmado</t>
+  </si>
+  <si>
+    <t>https://www.fadeeac.org.ar/wp-content/uploads/2026/10/1-Acuerdo-paritario-Sep-2026-Feb2027.pdf</t>
+  </si>
+  <si>
+    <t>Disposición DNRyRT 1277/2026: homologación del acuerdo del 18/9/2026</t>
+  </si>
+  <si>
+    <t>https://www.fadeeac.org.ar/wp-content/uploads/2026/10/Disp.-1277-26-Homolog.-paritaria-sep26-Feb27.pdf</t>
+  </si>
+  <si>
+    <t>Acuerdo del 18/9/2026: asignación extraordinaria no remunerativa de $1.200.000 (4 cuotas de $300.000 desde enero 2027)</t>
+  </si>
+  <si>
+    <t>https://www.fadeeac.org.ar/wp-content/uploads/2026/10/2-Acuerdo-Asignacion-Ext.No-Remunerativa.pdf</t>
+  </si>
+  <si>
     <t>Ley 23.041: Sueldo Anual Complementario</t>
   </si>
   <si>
@@ -581,6 +656,9 @@
   </si>
   <si>
     <t>Disposición DNRyRT 455/2026</t>
+  </si>
+  <si>
+    <t>Disposición DNRyRT 1277/2026</t>
   </si>
   <si>
     <t>Planilla de calcular.ar. Las actualizaciones del año están incluidas en el precio: cuando FADEEAC publica la planilla firmada de un mes nuevo, la cargamos y el mismo enlace de descarga te baja la versión al día.</t>
@@ -1436,7 +1514,7 @@
         <v>28</v>
       </c>
       <c r="D5">
-        <f>MATCH(B6,'Escala 2026'!$B$2:$G$2,0)</f>
+        <f>MATCH(B6,'Escala 2026'!$B$2:$M$2,0)</f>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
@@ -1447,7 +1525,7 @@
         <v>30</v>
       </c>
       <c r="D6">
-        <f>INDEX('Escala 2026'!$B$3:$G$11,MATCH(B5,'Escala 2026'!$A$3:$A$11,0),D5)</f>
+        <f>INDEX('Escala 2026'!$B$3:$M$11,MATCH(B5,'Escala 2026'!$A$3:$A$11,0),D5)</f>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
@@ -1671,10 +1749,10 @@
         <v>66</v>
       </c>
       <c r="B32" s="19">
-        <v>86.07469</v>
+        <v>90.09389</v>
       </c>
       <c r="C32" s="20">
-        <f>IF(B6="Agosto 2026","Valores de la planilla firmada de agosto 2026","Ojo: son los valores de agosto 2026. Reemplazalos por los de la planilla de "&amp;B6)</f>
+        <f>IF(B6="Octubre 2026","Valores de la planilla firmada de octubre 2026","Ojo: son los valores de octubre 2026. Reemplazalos por los de la planilla de "&amp;B6)</f>
       </c>
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.25">
@@ -1682,7 +1760,7 @@
         <v>67</v>
       </c>
       <c r="B33" s="14">
-        <v>16463.15</v>
+        <v>17231.89</v>
       </c>
       <c r="C33" s="20"/>
     </row>
@@ -1691,7 +1769,7 @@
         <v>68</v>
       </c>
       <c r="B34" s="14">
-        <v>8261.18</v>
+        <v>8646.93</v>
       </c>
       <c r="C34" s="20"/>
     </row>
@@ -1700,7 +1778,7 @@
         <v>69</v>
       </c>
       <c r="B35" s="14">
-        <v>19175</v>
+        <v>20070.36</v>
       </c>
       <c r="C35" s="20"/>
     </row>
@@ -1767,7 +1845,7 @@
       <formula1>"Chofer de Primera,Chofer de Segunda,Chofer de Tercera,Encargado,Peón,Ayudante mayor de 18 años,Oficial de Primera (taller),Oficial (taller),Medio Oficial (taller)"</formula1>
     </dataValidation>
     <dataValidation type="list" showErrorMessage="1" error="Elegí un mes de la lista." sqref="B6">
-      <formula1>"Marzo 2026,Abril 2026,Mayo 2026,Junio 2026,Julio 2026,Agosto 2026"</formula1>
+      <formula1>"Marzo 2026,Abril 2026,Mayo 2026,Junio 2026,Julio 2026,Agosto 2026,Septiembre 2026,Octubre 2026,Noviembre 2026,Diciembre 2026,Enero 2027,Febrero 2027"</formula1>
     </dataValidation>
     <dataValidation type="whole" allowBlank="1" showErrorMessage="1" error="Años enteros, de 0 a 60." sqref="B7">
       <formula1>0</formula1>
@@ -1961,7 +2039,7 @@
       <c r="J6" s="28"/>
       <c r="K6" s="28"/>
       <c r="L6" s="29">
-        <f>IF(B6="","",INDEX('Escala 2026'!$B$3:$G$11,MATCH(B6,'Escala 2026'!$A$3:$A$11,0),'Liquidador'!$D$5))</f>
+        <f>IF(B6="","",INDEX('Escala 2026'!$B$3:$M$11,MATCH(B6,'Escala 2026'!$A$3:$A$11,0),'Liquidador'!$D$5))</f>
       </c>
       <c r="M6" s="29">
         <f>IF(B6="","",E6*'Liquidador'!$B$32*T6)</f>
@@ -2001,7 +2079,7 @@
       <c r="J7" s="28"/>
       <c r="K7" s="28"/>
       <c r="L7" s="29">
-        <f>IF(B7="","",INDEX('Escala 2026'!$B$3:$G$11,MATCH(B7,'Escala 2026'!$A$3:$A$11,0),'Liquidador'!$D$5))</f>
+        <f>IF(B7="","",INDEX('Escala 2026'!$B$3:$M$11,MATCH(B7,'Escala 2026'!$A$3:$A$11,0),'Liquidador'!$D$5))</f>
       </c>
       <c r="M7" s="29">
         <f>IF(B7="","",E7*'Liquidador'!$B$32*T7)</f>
@@ -2041,7 +2119,7 @@
       <c r="J8" s="28"/>
       <c r="K8" s="28"/>
       <c r="L8" s="29">
-        <f>IF(B8="","",INDEX('Escala 2026'!$B$3:$G$11,MATCH(B8,'Escala 2026'!$A$3:$A$11,0),'Liquidador'!$D$5))</f>
+        <f>IF(B8="","",INDEX('Escala 2026'!$B$3:$M$11,MATCH(B8,'Escala 2026'!$A$3:$A$11,0),'Liquidador'!$D$5))</f>
       </c>
       <c r="M8" s="29">
         <f>IF(B8="","",E8*'Liquidador'!$B$32*T8)</f>
@@ -2081,7 +2159,7 @@
       <c r="J9" s="28"/>
       <c r="K9" s="28"/>
       <c r="L9" s="29">
-        <f>IF(B9="","",INDEX('Escala 2026'!$B$3:$G$11,MATCH(B9,'Escala 2026'!$A$3:$A$11,0),'Liquidador'!$D$5))</f>
+        <f>IF(B9="","",INDEX('Escala 2026'!$B$3:$M$11,MATCH(B9,'Escala 2026'!$A$3:$A$11,0),'Liquidador'!$D$5))</f>
       </c>
       <c r="M9" s="29">
         <f>IF(B9="","",E9*'Liquidador'!$B$32*T9)</f>
@@ -2121,7 +2199,7 @@
       <c r="J10" s="28"/>
       <c r="K10" s="28"/>
       <c r="L10" s="29">
-        <f>IF(B10="","",INDEX('Escala 2026'!$B$3:$G$11,MATCH(B10,'Escala 2026'!$A$3:$A$11,0),'Liquidador'!$D$5))</f>
+        <f>IF(B10="","",INDEX('Escala 2026'!$B$3:$M$11,MATCH(B10,'Escala 2026'!$A$3:$A$11,0),'Liquidador'!$D$5))</f>
       </c>
       <c r="M10" s="29">
         <f>IF(B10="","",E10*'Liquidador'!$B$32*T10)</f>
@@ -2161,7 +2239,7 @@
       <c r="J11" s="28"/>
       <c r="K11" s="28"/>
       <c r="L11" s="29">
-        <f>IF(B11="","",INDEX('Escala 2026'!$B$3:$G$11,MATCH(B11,'Escala 2026'!$A$3:$A$11,0),'Liquidador'!$D$5))</f>
+        <f>IF(B11="","",INDEX('Escala 2026'!$B$3:$M$11,MATCH(B11,'Escala 2026'!$A$3:$A$11,0),'Liquidador'!$D$5))</f>
       </c>
       <c r="M11" s="29">
         <f>IF(B11="","",E11*'Liquidador'!$B$32*T11)</f>
@@ -2201,7 +2279,7 @@
       <c r="J12" s="28"/>
       <c r="K12" s="28"/>
       <c r="L12" s="29">
-        <f>IF(B12="","",INDEX('Escala 2026'!$B$3:$G$11,MATCH(B12,'Escala 2026'!$A$3:$A$11,0),'Liquidador'!$D$5))</f>
+        <f>IF(B12="","",INDEX('Escala 2026'!$B$3:$M$11,MATCH(B12,'Escala 2026'!$A$3:$A$11,0),'Liquidador'!$D$5))</f>
       </c>
       <c r="M12" s="29">
         <f>IF(B12="","",E12*'Liquidador'!$B$32*T12)</f>
@@ -2241,7 +2319,7 @@
       <c r="J13" s="28"/>
       <c r="K13" s="28"/>
       <c r="L13" s="29">
-        <f>IF(B13="","",INDEX('Escala 2026'!$B$3:$G$11,MATCH(B13,'Escala 2026'!$A$3:$A$11,0),'Liquidador'!$D$5))</f>
+        <f>IF(B13="","",INDEX('Escala 2026'!$B$3:$M$11,MATCH(B13,'Escala 2026'!$A$3:$A$11,0),'Liquidador'!$D$5))</f>
       </c>
       <c r="M13" s="29">
         <f>IF(B13="","",E13*'Liquidador'!$B$32*T13)</f>
@@ -2281,7 +2359,7 @@
       <c r="J14" s="28"/>
       <c r="K14" s="28"/>
       <c r="L14" s="29">
-        <f>IF(B14="","",INDEX('Escala 2026'!$B$3:$G$11,MATCH(B14,'Escala 2026'!$A$3:$A$11,0),'Liquidador'!$D$5))</f>
+        <f>IF(B14="","",INDEX('Escala 2026'!$B$3:$M$11,MATCH(B14,'Escala 2026'!$A$3:$A$11,0),'Liquidador'!$D$5))</f>
       </c>
       <c r="M14" s="29">
         <f>IF(B14="","",E14*'Liquidador'!$B$32*T14)</f>
@@ -2321,7 +2399,7 @@
       <c r="J15" s="28"/>
       <c r="K15" s="28"/>
       <c r="L15" s="29">
-        <f>IF(B15="","",INDEX('Escala 2026'!$B$3:$G$11,MATCH(B15,'Escala 2026'!$A$3:$A$11,0),'Liquidador'!$D$5))</f>
+        <f>IF(B15="","",INDEX('Escala 2026'!$B$3:$M$11,MATCH(B15,'Escala 2026'!$A$3:$A$11,0),'Liquidador'!$D$5))</f>
       </c>
       <c r="M15" s="29">
         <f>IF(B15="","",E15*'Liquidador'!$B$32*T15)</f>
@@ -2361,7 +2439,7 @@
       <c r="J16" s="28"/>
       <c r="K16" s="28"/>
       <c r="L16" s="29">
-        <f>IF(B16="","",INDEX('Escala 2026'!$B$3:$G$11,MATCH(B16,'Escala 2026'!$A$3:$A$11,0),'Liquidador'!$D$5))</f>
+        <f>IF(B16="","",INDEX('Escala 2026'!$B$3:$M$11,MATCH(B16,'Escala 2026'!$A$3:$A$11,0),'Liquidador'!$D$5))</f>
       </c>
       <c r="M16" s="29">
         <f>IF(B16="","",E16*'Liquidador'!$B$32*T16)</f>
@@ -2401,7 +2479,7 @@
       <c r="J17" s="28"/>
       <c r="K17" s="28"/>
       <c r="L17" s="29">
-        <f>IF(B17="","",INDEX('Escala 2026'!$B$3:$G$11,MATCH(B17,'Escala 2026'!$A$3:$A$11,0),'Liquidador'!$D$5))</f>
+        <f>IF(B17="","",INDEX('Escala 2026'!$B$3:$M$11,MATCH(B17,'Escala 2026'!$A$3:$A$11,0),'Liquidador'!$D$5))</f>
       </c>
       <c r="M17" s="29">
         <f>IF(B17="","",E17*'Liquidador'!$B$32*T17)</f>
@@ -2441,7 +2519,7 @@
       <c r="J18" s="28"/>
       <c r="K18" s="28"/>
       <c r="L18" s="29">
-        <f>IF(B18="","",INDEX('Escala 2026'!$B$3:$G$11,MATCH(B18,'Escala 2026'!$A$3:$A$11,0),'Liquidador'!$D$5))</f>
+        <f>IF(B18="","",INDEX('Escala 2026'!$B$3:$M$11,MATCH(B18,'Escala 2026'!$A$3:$A$11,0),'Liquidador'!$D$5))</f>
       </c>
       <c r="M18" s="29">
         <f>IF(B18="","",E18*'Liquidador'!$B$32*T18)</f>
@@ -2481,7 +2559,7 @@
       <c r="J19" s="28"/>
       <c r="K19" s="28"/>
       <c r="L19" s="29">
-        <f>IF(B19="","",INDEX('Escala 2026'!$B$3:$G$11,MATCH(B19,'Escala 2026'!$A$3:$A$11,0),'Liquidador'!$D$5))</f>
+        <f>IF(B19="","",INDEX('Escala 2026'!$B$3:$M$11,MATCH(B19,'Escala 2026'!$A$3:$A$11,0),'Liquidador'!$D$5))</f>
       </c>
       <c r="M19" s="29">
         <f>IF(B19="","",E19*'Liquidador'!$B$32*T19)</f>
@@ -2521,7 +2599,7 @@
       <c r="J20" s="28"/>
       <c r="K20" s="28"/>
       <c r="L20" s="29">
-        <f>IF(B20="","",INDEX('Escala 2026'!$B$3:$G$11,MATCH(B20,'Escala 2026'!$A$3:$A$11,0),'Liquidador'!$D$5))</f>
+        <f>IF(B20="","",INDEX('Escala 2026'!$B$3:$M$11,MATCH(B20,'Escala 2026'!$A$3:$A$11,0),'Liquidador'!$D$5))</f>
       </c>
       <c r="M20" s="29">
         <f>IF(B20="","",E20*'Liquidador'!$B$32*T20)</f>
@@ -2561,7 +2639,7 @@
       <c r="J21" s="28"/>
       <c r="K21" s="28"/>
       <c r="L21" s="29">
-        <f>IF(B21="","",INDEX('Escala 2026'!$B$3:$G$11,MATCH(B21,'Escala 2026'!$A$3:$A$11,0),'Liquidador'!$D$5))</f>
+        <f>IF(B21="","",INDEX('Escala 2026'!$B$3:$M$11,MATCH(B21,'Escala 2026'!$A$3:$A$11,0),'Liquidador'!$D$5))</f>
       </c>
       <c r="M21" s="29">
         <f>IF(B21="","",E21*'Liquidador'!$B$32*T21)</f>
@@ -2601,7 +2679,7 @@
       <c r="J22" s="28"/>
       <c r="K22" s="28"/>
       <c r="L22" s="29">
-        <f>IF(B22="","",INDEX('Escala 2026'!$B$3:$G$11,MATCH(B22,'Escala 2026'!$A$3:$A$11,0),'Liquidador'!$D$5))</f>
+        <f>IF(B22="","",INDEX('Escala 2026'!$B$3:$M$11,MATCH(B22,'Escala 2026'!$A$3:$A$11,0),'Liquidador'!$D$5))</f>
       </c>
       <c r="M22" s="29">
         <f>IF(B22="","",E22*'Liquidador'!$B$32*T22)</f>
@@ -2641,7 +2719,7 @@
       <c r="J23" s="28"/>
       <c r="K23" s="28"/>
       <c r="L23" s="29">
-        <f>IF(B23="","",INDEX('Escala 2026'!$B$3:$G$11,MATCH(B23,'Escala 2026'!$A$3:$A$11,0),'Liquidador'!$D$5))</f>
+        <f>IF(B23="","",INDEX('Escala 2026'!$B$3:$M$11,MATCH(B23,'Escala 2026'!$A$3:$A$11,0),'Liquidador'!$D$5))</f>
       </c>
       <c r="M23" s="29">
         <f>IF(B23="","",E23*'Liquidador'!$B$32*T23)</f>
@@ -2681,7 +2759,7 @@
       <c r="J24" s="28"/>
       <c r="K24" s="28"/>
       <c r="L24" s="29">
-        <f>IF(B24="","",INDEX('Escala 2026'!$B$3:$G$11,MATCH(B24,'Escala 2026'!$A$3:$A$11,0),'Liquidador'!$D$5))</f>
+        <f>IF(B24="","",INDEX('Escala 2026'!$B$3:$M$11,MATCH(B24,'Escala 2026'!$A$3:$A$11,0),'Liquidador'!$D$5))</f>
       </c>
       <c r="M24" s="29">
         <f>IF(B24="","",E24*'Liquidador'!$B$32*T24)</f>
@@ -2721,7 +2799,7 @@
       <c r="J25" s="28"/>
       <c r="K25" s="28"/>
       <c r="L25" s="29">
-        <f>IF(B25="","",INDEX('Escala 2026'!$B$3:$G$11,MATCH(B25,'Escala 2026'!$A$3:$A$11,0),'Liquidador'!$D$5))</f>
+        <f>IF(B25="","",INDEX('Escala 2026'!$B$3:$M$11,MATCH(B25,'Escala 2026'!$A$3:$A$11,0),'Liquidador'!$D$5))</f>
       </c>
       <c r="M25" s="29">
         <f>IF(B25="","",E25*'Liquidador'!$B$32*T25)</f>
@@ -2761,7 +2839,7 @@
       <c r="J26" s="28"/>
       <c r="K26" s="28"/>
       <c r="L26" s="29">
-        <f>IF(B26="","",INDEX('Escala 2026'!$B$3:$G$11,MATCH(B26,'Escala 2026'!$A$3:$A$11,0),'Liquidador'!$D$5))</f>
+        <f>IF(B26="","",INDEX('Escala 2026'!$B$3:$M$11,MATCH(B26,'Escala 2026'!$A$3:$A$11,0),'Liquidador'!$D$5))</f>
       </c>
       <c r="M26" s="29">
         <f>IF(B26="","",E26*'Liquidador'!$B$32*T26)</f>
@@ -2801,7 +2879,7 @@
       <c r="J27" s="28"/>
       <c r="K27" s="28"/>
       <c r="L27" s="29">
-        <f>IF(B27="","",INDEX('Escala 2026'!$B$3:$G$11,MATCH(B27,'Escala 2026'!$A$3:$A$11,0),'Liquidador'!$D$5))</f>
+        <f>IF(B27="","",INDEX('Escala 2026'!$B$3:$M$11,MATCH(B27,'Escala 2026'!$A$3:$A$11,0),'Liquidador'!$D$5))</f>
       </c>
       <c r="M27" s="29">
         <f>IF(B27="","",E27*'Liquidador'!$B$32*T27)</f>
@@ -2841,7 +2919,7 @@
       <c r="J28" s="28"/>
       <c r="K28" s="28"/>
       <c r="L28" s="29">
-        <f>IF(B28="","",INDEX('Escala 2026'!$B$3:$G$11,MATCH(B28,'Escala 2026'!$A$3:$A$11,0),'Liquidador'!$D$5))</f>
+        <f>IF(B28="","",INDEX('Escala 2026'!$B$3:$M$11,MATCH(B28,'Escala 2026'!$A$3:$A$11,0),'Liquidador'!$D$5))</f>
       </c>
       <c r="M28" s="29">
         <f>IF(B28="","",E28*'Liquidador'!$B$32*T28)</f>
@@ -2881,7 +2959,7 @@
       <c r="J29" s="28"/>
       <c r="K29" s="28"/>
       <c r="L29" s="29">
-        <f>IF(B29="","",INDEX('Escala 2026'!$B$3:$G$11,MATCH(B29,'Escala 2026'!$A$3:$A$11,0),'Liquidador'!$D$5))</f>
+        <f>IF(B29="","",INDEX('Escala 2026'!$B$3:$M$11,MATCH(B29,'Escala 2026'!$A$3:$A$11,0),'Liquidador'!$D$5))</f>
       </c>
       <c r="M29" s="29">
         <f>IF(B29="","",E29*'Liquidador'!$B$32*T29)</f>
@@ -2921,7 +2999,7 @@
       <c r="J30" s="28"/>
       <c r="K30" s="28"/>
       <c r="L30" s="29">
-        <f>IF(B30="","",INDEX('Escala 2026'!$B$3:$G$11,MATCH(B30,'Escala 2026'!$A$3:$A$11,0),'Liquidador'!$D$5))</f>
+        <f>IF(B30="","",INDEX('Escala 2026'!$B$3:$M$11,MATCH(B30,'Escala 2026'!$A$3:$A$11,0),'Liquidador'!$D$5))</f>
       </c>
       <c r="M30" s="29">
         <f>IF(B30="","",E30*'Liquidador'!$B$32*T30)</f>
@@ -2961,7 +3039,7 @@
       <c r="J31" s="28"/>
       <c r="K31" s="28"/>
       <c r="L31" s="29">
-        <f>IF(B31="","",INDEX('Escala 2026'!$B$3:$G$11,MATCH(B31,'Escala 2026'!$A$3:$A$11,0),'Liquidador'!$D$5))</f>
+        <f>IF(B31="","",INDEX('Escala 2026'!$B$3:$M$11,MATCH(B31,'Escala 2026'!$A$3:$A$11,0),'Liquidador'!$D$5))</f>
       </c>
       <c r="M31" s="29">
         <f>IF(B31="","",E31*'Liquidador'!$B$32*T31)</f>
@@ -3001,7 +3079,7 @@
       <c r="J32" s="28"/>
       <c r="K32" s="28"/>
       <c r="L32" s="29">
-        <f>IF(B32="","",INDEX('Escala 2026'!$B$3:$G$11,MATCH(B32,'Escala 2026'!$A$3:$A$11,0),'Liquidador'!$D$5))</f>
+        <f>IF(B32="","",INDEX('Escala 2026'!$B$3:$M$11,MATCH(B32,'Escala 2026'!$A$3:$A$11,0),'Liquidador'!$D$5))</f>
       </c>
       <c r="M32" s="29">
         <f>IF(B32="","",E32*'Liquidador'!$B$32*T32)</f>
@@ -3041,7 +3119,7 @@
       <c r="J33" s="28"/>
       <c r="K33" s="28"/>
       <c r="L33" s="29">
-        <f>IF(B33="","",INDEX('Escala 2026'!$B$3:$G$11,MATCH(B33,'Escala 2026'!$A$3:$A$11,0),'Liquidador'!$D$5))</f>
+        <f>IF(B33="","",INDEX('Escala 2026'!$B$3:$M$11,MATCH(B33,'Escala 2026'!$A$3:$A$11,0),'Liquidador'!$D$5))</f>
       </c>
       <c r="M33" s="29">
         <f>IF(B33="","",E33*'Liquidador'!$B$32*T33)</f>
@@ -3081,7 +3159,7 @@
       <c r="J34" s="28"/>
       <c r="K34" s="28"/>
       <c r="L34" s="29">
-        <f>IF(B34="","",INDEX('Escala 2026'!$B$3:$G$11,MATCH(B34,'Escala 2026'!$A$3:$A$11,0),'Liquidador'!$D$5))</f>
+        <f>IF(B34="","",INDEX('Escala 2026'!$B$3:$M$11,MATCH(B34,'Escala 2026'!$A$3:$A$11,0),'Liquidador'!$D$5))</f>
       </c>
       <c r="M34" s="29">
         <f>IF(B34="","",E34*'Liquidador'!$B$32*T34)</f>
@@ -3121,7 +3199,7 @@
       <c r="J35" s="28"/>
       <c r="K35" s="28"/>
       <c r="L35" s="29">
-        <f>IF(B35="","",INDEX('Escala 2026'!$B$3:$G$11,MATCH(B35,'Escala 2026'!$A$3:$A$11,0),'Liquidador'!$D$5))</f>
+        <f>IF(B35="","",INDEX('Escala 2026'!$B$3:$M$11,MATCH(B35,'Escala 2026'!$A$3:$A$11,0),'Liquidador'!$D$5))</f>
       </c>
       <c r="M35" s="29">
         <f>IF(B35="","",E35*'Liquidador'!$B$32*T35)</f>
@@ -3759,14 +3837,14 @@
   <sheetPr>
     <tabColor rgb="FF1565C0"/>
   </sheetPr>
-  <dimension ref="A1:G21"/>
+  <dimension ref="A1:M27"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="32" customWidth="1"/>
-    <col min="2" max="7" width="16" customWidth="1"/>
+    <col min="2" max="13" width="16" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="28" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" ht="28" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1" s="49" t="s">
         <v>136</v>
       </c>
@@ -3776,8 +3854,14 @@
       <c r="E1" s="49"/>
       <c r="F1" s="49"/>
       <c r="G1" s="49"/>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H1" s="49"/>
+      <c r="I1" s="49"/>
+      <c r="J1" s="49"/>
+      <c r="K1" s="49"/>
+      <c r="L1" s="49"/>
+      <c r="M1" s="49"/>
+    </row>
+    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A2" s="50" t="s">
         <v>27</v>
       </c>
@@ -3797,10 +3881,28 @@
         <v>141</v>
       </c>
       <c r="G2" s="50" t="s">
+        <v>142</v>
+      </c>
+      <c r="H2" s="50" t="s">
+        <v>143</v>
+      </c>
+      <c r="I2" s="50" t="s">
+        <v>144</v>
+      </c>
+      <c r="J2" s="50" t="s">
+        <v>145</v>
+      </c>
+      <c r="K2" s="50" t="s">
+        <v>146</v>
+      </c>
+      <c r="L2" s="50" t="s">
+        <v>147</v>
+      </c>
+      <c r="M2" s="50" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A3" s="51" t="s">
         <v>28</v>
       </c>
@@ -3822,10 +3924,28 @@
       <c r="G3" s="52">
         <v>1075910.44</v>
       </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H3" s="52">
+        <v>1095276.83</v>
+      </c>
+      <c r="I3" s="52">
+        <v>1126149.4</v>
+      </c>
+      <c r="J3" s="52">
+        <v>1145293.94</v>
+      </c>
+      <c r="K3" s="52">
+        <v>1163618.64</v>
+      </c>
+      <c r="L3" s="52">
+        <v>1182236.54</v>
+      </c>
+      <c r="M3" s="52">
+        <v>1199970.09</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A4" s="53" t="s">
-        <v>142</v>
+        <v>148</v>
       </c>
       <c r="B4" s="54">
         <v>901112.88</v>
@@ -3845,10 +3965,28 @@
       <c r="G4" s="54">
         <v>1056737.31</v>
       </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H4" s="54">
+        <v>1075758.58</v>
+      </c>
+      <c r="I4" s="54">
+        <v>1106080.99</v>
+      </c>
+      <c r="J4" s="54">
+        <v>1124884.37</v>
+      </c>
+      <c r="K4" s="54">
+        <v>1142882.52</v>
+      </c>
+      <c r="L4" s="54">
+        <v>1161168.64</v>
+      </c>
+      <c r="M4" s="54">
+        <v>1178586.17</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A5" s="51" t="s">
-        <v>143</v>
+        <v>149</v>
       </c>
       <c r="B5" s="52">
         <v>884746.81</v>
@@ -3868,10 +4006,28 @@
       <c r="G5" s="52">
         <v>1037544.76</v>
       </c>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H5" s="52">
+        <v>1056220.57</v>
+      </c>
+      <c r="I5" s="52">
+        <v>1085992.26</v>
+      </c>
+      <c r="J5" s="52">
+        <v>1104454.13</v>
+      </c>
+      <c r="K5" s="52">
+        <v>1122125.4</v>
+      </c>
+      <c r="L5" s="52">
+        <v>1140079.41</v>
+      </c>
+      <c r="M5" s="52">
+        <v>1157180.6</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A6" s="53" t="s">
-        <v>144</v>
+        <v>150</v>
       </c>
       <c r="B6" s="54">
         <v>862285.2</v>
@@ -3891,10 +4047,28 @@
       <c r="G6" s="54">
         <v>1011203.97</v>
       </c>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H6" s="54">
+        <v>1029405.64</v>
+      </c>
+      <c r="I6" s="54">
+        <v>1058421.5</v>
+      </c>
+      <c r="J6" s="54">
+        <v>1076414.67</v>
+      </c>
+      <c r="K6" s="54">
+        <v>1093637.3</v>
+      </c>
+      <c r="L6" s="54">
+        <v>1111135.5</v>
+      </c>
+      <c r="M6" s="54">
+        <v>1127802.53</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A7" s="51" t="s">
-        <v>145</v>
+        <v>151</v>
       </c>
       <c r="B7" s="52">
         <v>837929.46</v>
@@ -3914,10 +4088,28 @@
       <c r="G7" s="52">
         <v>982641.94</v>
       </c>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H7" s="52">
+        <v>1000329.49</v>
+      </c>
+      <c r="I7" s="52">
+        <v>1028525.78</v>
+      </c>
+      <c r="J7" s="52">
+        <v>1046010.72</v>
+      </c>
+      <c r="K7" s="52">
+        <v>1062746.89</v>
+      </c>
+      <c r="L7" s="52">
+        <v>1079750.84</v>
+      </c>
+      <c r="M7" s="52">
+        <v>1095947.1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A8" s="53" t="s">
-        <v>146</v>
+        <v>152</v>
       </c>
       <c r="B8" s="54">
         <v>821870.69</v>
@@ -3937,10 +4129,28 @@
       <c r="G8" s="54">
         <v>963809.78</v>
       </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H8" s="54">
+        <v>981158.36</v>
+      </c>
+      <c r="I8" s="54">
+        <v>1008814.27</v>
+      </c>
+      <c r="J8" s="54">
+        <v>1025964.11</v>
+      </c>
+      <c r="K8" s="54">
+        <v>1042379.54</v>
+      </c>
+      <c r="L8" s="54">
+        <v>1059057.61</v>
+      </c>
+      <c r="M8" s="54">
+        <v>1074943.47</v>
+      </c>
+    </row>
+    <row r="9" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A9" s="51" t="s">
-        <v>147</v>
+        <v>153</v>
       </c>
       <c r="B9" s="52">
         <v>1021805.24</v>
@@ -3960,10 +4170,28 @@
       <c r="G9" s="52">
         <v>1198273.54</v>
       </c>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H9" s="52">
+        <v>1219842.46</v>
+      </c>
+      <c r="I9" s="52">
+        <v>1254226.16</v>
+      </c>
+      <c r="J9" s="52">
+        <v>1275548</v>
+      </c>
+      <c r="K9" s="52">
+        <v>1295956.77</v>
+      </c>
+      <c r="L9" s="52">
+        <v>1316692.08</v>
+      </c>
+      <c r="M9" s="52">
+        <v>1336442.46</v>
+      </c>
+    </row>
+    <row r="10" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A10" s="53" t="s">
-        <v>148</v>
+        <v>154</v>
       </c>
       <c r="B10" s="54">
         <v>921140.39</v>
@@ -3983,10 +4211,28 @@
       <c r="G10" s="54">
         <v>1080223.62</v>
       </c>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H10" s="54">
+        <v>1099667.65</v>
+      </c>
+      <c r="I10" s="54">
+        <v>1130663.98</v>
+      </c>
+      <c r="J10" s="54">
+        <v>1149885.27</v>
+      </c>
+      <c r="K10" s="54">
+        <v>1168283.43</v>
+      </c>
+      <c r="L10" s="54">
+        <v>1186975.96</v>
+      </c>
+      <c r="M10" s="54">
+        <v>1204780.6</v>
+      </c>
+    </row>
+    <row r="11" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A11" s="51" t="s">
-        <v>149</v>
+        <v>155</v>
       </c>
       <c r="B11" s="52">
         <v>870164.95</v>
@@ -4006,10 +4252,28 @@
       <c r="G11" s="52">
         <v>1020444.59</v>
       </c>
-    </row>
-    <row r="13" ht="28" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H11" s="52">
+        <v>1038812.59</v>
+      </c>
+      <c r="I11" s="52">
+        <v>1068093.6</v>
+      </c>
+      <c r="J11" s="52">
+        <v>1086251.19</v>
+      </c>
+      <c r="K11" s="52">
+        <v>1103631.21</v>
+      </c>
+      <c r="L11" s="52">
+        <v>1121289.31</v>
+      </c>
+      <c r="M11" s="52">
+        <v>1138108.65</v>
+      </c>
+    </row>
+    <row r="13" ht="28" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A13" s="6" t="s">
-        <v>150</v>
+        <v>156</v>
       </c>
       <c r="B13" s="6"/>
       <c r="C13" s="6"/>
@@ -4017,10 +4281,16 @@
       <c r="E13" s="6"/>
       <c r="F13" s="6"/>
       <c r="G13" s="6"/>
-    </row>
-    <row r="14" ht="28" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H13" s="6"/>
+      <c r="I13" s="6"/>
+      <c r="J13" s="6"/>
+      <c r="K13" s="6"/>
+      <c r="L13" s="6"/>
+      <c r="M13" s="6"/>
+    </row>
+    <row r="14" ht="28" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A14" s="6" t="s">
-        <v>151</v>
+        <v>157</v>
       </c>
       <c r="B14" s="6"/>
       <c r="C14" s="6"/>
@@ -4028,10 +4298,16 @@
       <c r="E14" s="6"/>
       <c r="F14" s="6"/>
       <c r="G14" s="6"/>
-    </row>
-    <row r="15" ht="28" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H14" s="6"/>
+      <c r="I14" s="6"/>
+      <c r="J14" s="6"/>
+      <c r="K14" s="6"/>
+      <c r="L14" s="6"/>
+      <c r="M14" s="6"/>
+    </row>
+    <row r="15" ht="28" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A15" s="6" t="s">
-        <v>152</v>
+        <v>158</v>
       </c>
       <c r="B15" s="6"/>
       <c r="C15" s="6"/>
@@ -4039,10 +4315,16 @@
       <c r="E15" s="6"/>
       <c r="F15" s="6"/>
       <c r="G15" s="6"/>
-    </row>
-    <row r="16" ht="28" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H15" s="6"/>
+      <c r="I15" s="6"/>
+      <c r="J15" s="6"/>
+      <c r="K15" s="6"/>
+      <c r="L15" s="6"/>
+      <c r="M15" s="6"/>
+    </row>
+    <row r="16" ht="28" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A16" s="6" t="s">
-        <v>153</v>
+        <v>159</v>
       </c>
       <c r="B16" s="6"/>
       <c r="C16" s="6"/>
@@ -4050,10 +4332,16 @@
       <c r="E16" s="6"/>
       <c r="F16" s="6"/>
       <c r="G16" s="6"/>
-    </row>
-    <row r="17" ht="28" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H16" s="6"/>
+      <c r="I16" s="6"/>
+      <c r="J16" s="6"/>
+      <c r="K16" s="6"/>
+      <c r="L16" s="6"/>
+      <c r="M16" s="6"/>
+    </row>
+    <row r="17" ht="28" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A17" s="6" t="s">
-        <v>154</v>
+        <v>160</v>
       </c>
       <c r="B17" s="6"/>
       <c r="C17" s="6"/>
@@ -4061,10 +4349,16 @@
       <c r="E17" s="6"/>
       <c r="F17" s="6"/>
       <c r="G17" s="6"/>
-    </row>
-    <row r="18" ht="28" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H17" s="6"/>
+      <c r="I17" s="6"/>
+      <c r="J17" s="6"/>
+      <c r="K17" s="6"/>
+      <c r="L17" s="6"/>
+      <c r="M17" s="6"/>
+    </row>
+    <row r="18" ht="28" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A18" s="6" t="s">
-        <v>155</v>
+        <v>161</v>
       </c>
       <c r="B18" s="6"/>
       <c r="C18" s="6"/>
@@ -4072,10 +4366,33 @@
       <c r="E18" s="6"/>
       <c r="F18" s="6"/>
       <c r="G18" s="6"/>
-    </row>
-    <row r="20" ht="30" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H18" s="6"/>
+      <c r="I18" s="6"/>
+      <c r="J18" s="6"/>
+      <c r="K18" s="6"/>
+      <c r="L18" s="6"/>
+      <c r="M18" s="6"/>
+    </row>
+    <row r="19" ht="28" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A19" s="6" t="s">
+        <v>162</v>
+      </c>
+      <c r="B19" s="6"/>
+      <c r="C19" s="6"/>
+      <c r="D19" s="6"/>
+      <c r="E19" s="6"/>
+      <c r="F19" s="6"/>
+      <c r="G19" s="6"/>
+      <c r="H19" s="6"/>
+      <c r="I19" s="6"/>
+      <c r="J19" s="6"/>
+      <c r="K19" s="6"/>
+      <c r="L19" s="6"/>
+      <c r="M19" s="6"/>
+    </row>
+    <row r="20" ht="28" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A20" s="6" t="s">
-        <v>156</v>
+        <v>163</v>
       </c>
       <c r="B20" s="6"/>
       <c r="C20" s="6"/>
@@ -4083,10 +4400,16 @@
       <c r="E20" s="6"/>
       <c r="F20" s="6"/>
       <c r="G20" s="6"/>
-    </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H20" s="6"/>
+      <c r="I20" s="6"/>
+      <c r="J20" s="6"/>
+      <c r="K20" s="6"/>
+      <c r="L20" s="6"/>
+      <c r="M20" s="6"/>
+    </row>
+    <row r="21" ht="28" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A21" s="6" t="s">
-        <v>157</v>
+        <v>164</v>
       </c>
       <c r="B21" s="6"/>
       <c r="C21" s="6"/>
@@ -4094,18 +4417,115 @@
       <c r="E21" s="6"/>
       <c r="F21" s="6"/>
       <c r="G21" s="6"/>
+      <c r="H21" s="6"/>
+      <c r="I21" s="6"/>
+      <c r="J21" s="6"/>
+      <c r="K21" s="6"/>
+      <c r="L21" s="6"/>
+      <c r="M21" s="6"/>
+    </row>
+    <row r="22" ht="28" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A22" s="6" t="s">
+        <v>165</v>
+      </c>
+      <c r="B22" s="6"/>
+      <c r="C22" s="6"/>
+      <c r="D22" s="6"/>
+      <c r="E22" s="6"/>
+      <c r="F22" s="6"/>
+      <c r="G22" s="6"/>
+      <c r="H22" s="6"/>
+      <c r="I22" s="6"/>
+      <c r="J22" s="6"/>
+      <c r="K22" s="6"/>
+      <c r="L22" s="6"/>
+      <c r="M22" s="6"/>
+    </row>
+    <row r="23" ht="28" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A23" s="6" t="s">
+        <v>166</v>
+      </c>
+      <c r="B23" s="6"/>
+      <c r="C23" s="6"/>
+      <c r="D23" s="6"/>
+      <c r="E23" s="6"/>
+      <c r="F23" s="6"/>
+      <c r="G23" s="6"/>
+      <c r="H23" s="6"/>
+      <c r="I23" s="6"/>
+      <c r="J23" s="6"/>
+      <c r="K23" s="6"/>
+      <c r="L23" s="6"/>
+      <c r="M23" s="6"/>
+    </row>
+    <row r="24" ht="28" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A24" s="6" t="s">
+        <v>167</v>
+      </c>
+      <c r="B24" s="6"/>
+      <c r="C24" s="6"/>
+      <c r="D24" s="6"/>
+      <c r="E24" s="6"/>
+      <c r="F24" s="6"/>
+      <c r="G24" s="6"/>
+      <c r="H24" s="6"/>
+      <c r="I24" s="6"/>
+      <c r="J24" s="6"/>
+      <c r="K24" s="6"/>
+      <c r="L24" s="6"/>
+      <c r="M24" s="6"/>
+    </row>
+    <row r="26" ht="30" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A26" s="6" t="s">
+        <v>168</v>
+      </c>
+      <c r="B26" s="6"/>
+      <c r="C26" s="6"/>
+      <c r="D26" s="6"/>
+      <c r="E26" s="6"/>
+      <c r="F26" s="6"/>
+      <c r="G26" s="6"/>
+      <c r="H26" s="6"/>
+      <c r="I26" s="6"/>
+      <c r="J26" s="6"/>
+      <c r="K26" s="6"/>
+      <c r="L26" s="6"/>
+      <c r="M26" s="6"/>
+    </row>
+    <row r="27" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A27" s="6" t="s">
+        <v>169</v>
+      </c>
+      <c r="B27" s="6"/>
+      <c r="C27" s="6"/>
+      <c r="D27" s="6"/>
+      <c r="E27" s="6"/>
+      <c r="F27" s="6"/>
+      <c r="G27" s="6"/>
+      <c r="H27" s="6"/>
+      <c r="I27" s="6"/>
+      <c r="J27" s="6"/>
+      <c r="K27" s="6"/>
+      <c r="L27" s="6"/>
+      <c r="M27" s="6"/>
     </row>
   </sheetData>
-  <mergeCells count="9">
-    <mergeCell ref="A1:G1"/>
-    <mergeCell ref="A13:G13"/>
-    <mergeCell ref="A14:G14"/>
-    <mergeCell ref="A15:G15"/>
-    <mergeCell ref="A16:G16"/>
-    <mergeCell ref="A17:G17"/>
-    <mergeCell ref="A18:G18"/>
-    <mergeCell ref="A20:G20"/>
-    <mergeCell ref="A21:G21"/>
+  <mergeCells count="15">
+    <mergeCell ref="A1:M1"/>
+    <mergeCell ref="A13:M13"/>
+    <mergeCell ref="A14:M14"/>
+    <mergeCell ref="A15:M15"/>
+    <mergeCell ref="A16:M16"/>
+    <mergeCell ref="A17:M17"/>
+    <mergeCell ref="A18:M18"/>
+    <mergeCell ref="A19:M19"/>
+    <mergeCell ref="A20:M20"/>
+    <mergeCell ref="A21:M21"/>
+    <mergeCell ref="A22:M22"/>
+    <mergeCell ref="A23:M23"/>
+    <mergeCell ref="A24:M24"/>
+    <mergeCell ref="A26:M26"/>
+    <mergeCell ref="A27:M27"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
@@ -4117,7 +4537,7 @@
   <sheetPr>
     <tabColor rgb="FF37474F"/>
   </sheetPr>
-  <dimension ref="A1:B21"/>
+  <dimension ref="A1:B31"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="62" customWidth="1"/>
@@ -4126,143 +4546,222 @@
   <sheetData>
     <row r="1" ht="28" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="55" t="s">
-        <v>158</v>
+        <v>170</v>
       </c>
       <c r="B1" s="55"/>
     </row>
     <row r="2" ht="30" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="56" t="s">
-        <v>159</v>
+        <v>171</v>
       </c>
       <c r="B2" s="56"/>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="57" t="s">
-        <v>160</v>
+        <v>172</v>
       </c>
       <c r="B4" s="57" t="s">
-        <v>161</v>
+        <v>173</v>
       </c>
     </row>
     <row r="5" ht="32" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="58" t="s">
-        <v>162</v>
+        <v>174</v>
       </c>
       <c r="B5" s="59" t="s">
-        <v>163</v>
+        <v>175</v>
       </c>
     </row>
     <row r="6" ht="32" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" s="60" t="s">
-        <v>164</v>
+        <v>176</v>
       </c>
       <c r="B6" s="61" t="s">
-        <v>165</v>
+        <v>177</v>
       </c>
     </row>
     <row r="7" ht="32" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" s="58" t="s">
-        <v>166</v>
+        <v>178</v>
       </c>
       <c r="B7" s="59" t="s">
-        <v>167</v>
+        <v>179</v>
       </c>
     </row>
     <row r="8" ht="32" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" s="60" t="s">
-        <v>168</v>
+        <v>180</v>
       </c>
       <c r="B8" s="61" t="s">
-        <v>169</v>
+        <v>181</v>
       </c>
     </row>
     <row r="9" ht="32" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" s="58" t="s">
-        <v>170</v>
+        <v>182</v>
       </c>
       <c r="B9" s="59" t="s">
-        <v>171</v>
+        <v>183</v>
       </c>
     </row>
     <row r="10" ht="32" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" s="60" t="s">
-        <v>172</v>
+        <v>184</v>
       </c>
       <c r="B10" s="61" t="s">
-        <v>173</v>
+        <v>185</v>
       </c>
     </row>
     <row r="11" ht="32" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" s="58" t="s">
-        <v>174</v>
+        <v>186</v>
       </c>
       <c r="B11" s="59" t="s">
-        <v>173</v>
+        <v>187</v>
       </c>
     </row>
     <row r="12" ht="32" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" s="60" t="s">
-        <v>175</v>
+        <v>188</v>
       </c>
       <c r="B12" s="61" t="s">
-        <v>176</v>
+        <v>187</v>
       </c>
     </row>
     <row r="13" ht="32" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" s="58" t="s">
-        <v>177</v>
+        <v>189</v>
       </c>
       <c r="B13" s="59" t="s">
-        <v>178</v>
+        <v>187</v>
       </c>
     </row>
     <row r="14" ht="32" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" s="60" t="s">
-        <v>179</v>
+        <v>190</v>
       </c>
       <c r="B14" s="61" t="s">
-        <v>180</v>
+        <v>187</v>
       </c>
     </row>
     <row r="15" ht="32" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" s="58" t="s">
-        <v>181</v>
+        <v>191</v>
       </c>
       <c r="B15" s="59" t="s">
-        <v>182</v>
+        <v>187</v>
       </c>
     </row>
     <row r="16" ht="32" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" s="60" t="s">
-        <v>183</v>
+        <v>192</v>
       </c>
       <c r="B16" s="61" t="s">
-        <v>184</v>
-      </c>
-    </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A18" s="62" t="s">
-        <v>185</v>
-      </c>
-    </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A19" s="6" t="s">
-        <v>186</v>
-      </c>
-      <c r="B19" s="6"/>
-    </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A21" s="6" t="s">
         <v>187</v>
       </c>
-      <c r="B21" s="6"/>
+    </row>
+    <row r="17" ht="32" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A17" s="58" t="s">
+        <v>193</v>
+      </c>
+      <c r="B17" s="59" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="18" ht="32" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A18" s="60" t="s">
+        <v>194</v>
+      </c>
+      <c r="B18" s="61" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="19" ht="32" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A19" s="58" t="s">
+        <v>196</v>
+      </c>
+      <c r="B19" s="59" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="20" ht="32" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A20" s="60" t="s">
+        <v>198</v>
+      </c>
+      <c r="B20" s="61" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="21" ht="32" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A21" s="58" t="s">
+        <v>200</v>
+      </c>
+      <c r="B21" s="59" t="s">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="22" ht="32" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A22" s="60" t="s">
+        <v>202</v>
+      </c>
+      <c r="B22" s="61" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="23" ht="32" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A23" s="58" t="s">
+        <v>204</v>
+      </c>
+      <c r="B23" s="59" t="s">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="24" ht="32" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A24" s="60" t="s">
+        <v>206</v>
+      </c>
+      <c r="B24" s="61" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="25" ht="32" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A25" s="58" t="s">
+        <v>208</v>
+      </c>
+      <c r="B25" s="59" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="27" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A27" s="62" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A28" s="6" t="s">
+        <v>211</v>
+      </c>
+      <c r="B28" s="6"/>
+    </row>
+    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A29" s="6" t="s">
+        <v>212</v>
+      </c>
+      <c r="B29" s="6"/>
+    </row>
+    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A31" s="6" t="s">
+        <v>213</v>
+      </c>
+      <c r="B31" s="6"/>
     </row>
   </sheetData>
-  <mergeCells count="4">
+  <mergeCells count="5">
     <mergeCell ref="A1:B1"/>
     <mergeCell ref="A2:B2"/>
-    <mergeCell ref="A19:B19"/>
-    <mergeCell ref="A21:B21"/>
+    <mergeCell ref="A28:B28"/>
+    <mergeCell ref="A29:B29"/>
+    <mergeCell ref="A31:B31"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="B5" r:id="rId1"/>
@@ -4277,6 +4776,15 @@
     <hyperlink ref="B14" r:id="rId10"/>
     <hyperlink ref="B15" r:id="rId11"/>
     <hyperlink ref="B16" r:id="rId12"/>
+    <hyperlink ref="B17" r:id="rId13"/>
+    <hyperlink ref="B18" r:id="rId14"/>
+    <hyperlink ref="B19" r:id="rId15"/>
+    <hyperlink ref="B20" r:id="rId16"/>
+    <hyperlink ref="B21" r:id="rId17"/>
+    <hyperlink ref="B22" r:id="rId18"/>
+    <hyperlink ref="B23" r:id="rId19"/>
+    <hyperlink ref="B24" r:id="rId20"/>
+    <hyperlink ref="B25" r:id="rId21"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>